<commit_message>
Corrida | ARG-ESS | 2026-03-26 14:45:36.49389
</commit_message>
<xml_diff>
--- a/indicadores/ARG-ESS_out.xlsx
+++ b/indicadores/ARG-ESS_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">25/03/2026</t>
+    <t xml:space="preserve">26/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1235,7 +1235,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.602000954237363</v>
+        <v>0.601501539331679</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1293,7 +1293,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.362405148902696</v>
+        <v>0.361804101818379</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1363,7 +1363,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00443934477492296</v>
+        <v>0.00398766920287295</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1393,7 +1393,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.872886719811067</v>
+        <v>0.867273272632357</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -9786,7 +9786,7 @@
         <v>220</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0815979852971059</v>
+        <v>-0.0812621140331287</v>
       </c>
     </row>
     <row r="6">
@@ -9794,7 +9794,7 @@
         <v>221</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0407428209864884</v>
+        <v>0.0399445287858748</v>
       </c>
     </row>
     <row r="7">
@@ -9802,7 +9802,7 @@
         <v>222</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.237940744114264</v>
+        <v>0.236943660235123</v>
       </c>
     </row>
     <row r="8">
@@ -9810,7 +9810,7 @@
         <v>223</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.459336174439361</v>
+        <v>0.458798346550569</v>
       </c>
     </row>
     <row r="9">
@@ -9818,7 +9818,7 @@
         <v>224</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.602000954237363</v>
+        <v>0.601501539331679</v>
       </c>
     </row>
     <row r="10">
@@ -9826,7 +9826,7 @@
         <v>225</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.569511480077779</v>
+        <v>0.569256970325015</v>
       </c>
     </row>
     <row r="11">
@@ -9834,7 +9834,7 @@
         <v>226</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.402312998981605</v>
+        <v>0.402295996359951</v>
       </c>
     </row>
     <row r="12">
@@ -9842,7 +9842,7 @@
         <v>227</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.224930587462334</v>
+        <v>0.225080821265488</v>
       </c>
     </row>
     <row r="13">
@@ -9850,7 +9850,7 @@
         <v>228</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.104548935264558</v>
+        <v>0.105141084266131</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | ARG-ESS | 2026-03-26 15:10:39.15172
</commit_message>
<xml_diff>
--- a/indicadores/ARG-ESS_out.xlsx
+++ b/indicadores/ARG-ESS_out.xlsx
@@ -1235,7 +1235,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.601501539331679</v>
+        <v>0.601910742305836</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1293,7 +1293,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.361804101818379</v>
+        <v>0.362296541703163</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1363,7 +1363,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00398766920287295</v>
+        <v>0.00395619748110876</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1393,7 +1393,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.867273272632357</v>
+        <v>0.866596808626046</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -9786,7 +9786,7 @@
         <v>220</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0812621140331287</v>
+        <v>-0.0810352050436087</v>
       </c>
     </row>
     <row r="6">
@@ -9794,7 +9794,7 @@
         <v>221</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0399445287858748</v>
+        <v>0.0402500140844762</v>
       </c>
     </row>
     <row r="7">
@@ -9802,7 +9802,7 @@
         <v>222</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.236943660235123</v>
+        <v>0.236767051253355</v>
       </c>
     </row>
     <row r="8">
@@ -9810,7 +9810,7 @@
         <v>223</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.458798346550569</v>
+        <v>0.458724293738252</v>
       </c>
     </row>
     <row r="9">
@@ -9818,7 +9818,7 @@
         <v>224</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.601501539331679</v>
+        <v>0.601910742305836</v>
       </c>
     </row>
     <row r="10">
@@ -9826,7 +9826,7 @@
         <v>225</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.569256970325015</v>
+        <v>0.569788141883</v>
       </c>
     </row>
     <row r="11">
@@ -9834,7 +9834,7 @@
         <v>226</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.402295996359951</v>
+        <v>0.402808807113062</v>
       </c>
     </row>
     <row r="12">
@@ -9842,7 +9842,7 @@
         <v>227</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.225080821265488</v>
+        <v>0.22543289538925</v>
       </c>
     </row>
     <row r="13">
@@ -9850,7 +9850,7 @@
         <v>228</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.105141084266131</v>
+        <v>0.10540561531832</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | ARG-ESS | 2026-03-30 11:32:04.328412
</commit_message>
<xml_diff>
--- a/indicadores/ARG-ESS_out.xlsx
+++ b/indicadores/ARG-ESS_out.xlsx
@@ -9908,4 +9908,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64EE0691-6624-4D5D-990D-043CFB93874C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{319E09E3-5999-4BA9-AE4E-1088A538FE25}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A42C381E-09B7-4873-8485-7490A963766E}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-ESS | 2026-06-17 11:53:48.138992
</commit_message>
<xml_diff>
--- a/indicadores/ARG-ESS_out.xlsx
+++ b/indicadores/ARG-ESS_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="231">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Egresos por servicios de Argentina</t>
+    <t xml:space="preserve">Egresos por servicios</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentina</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">30/03/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1203,9 +1209,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1216,7 +1226,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1230,12 +1240,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.579327025860819</v>
+        <v>0.577296261064304</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1246,7 +1256,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1274,7 +1284,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1288,12 +1298,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.335619802892742</v>
+        <v>0.333270973038825</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1316,7 +1326,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1330,7 +1340,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1344,7 +1354,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1358,12 +1368,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0050691223722586</v>
+        <v>0.00935338540452576</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1374,7 +1384,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1388,12 +1398,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.821075588484585</v>
+        <v>0.800563499721089</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1536,10 +1546,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1552,10 +1562,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1579,66 +1589,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2241.8</v>
@@ -1691,7 +1701,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1494.9</v>
@@ -1748,7 +1758,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>1621.6</v>
@@ -1805,7 +1815,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1784.8</v>
@@ -1862,7 +1872,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2322.2</v>
@@ -1921,7 +1931,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1565.8</v>
@@ -1980,7 +1990,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1627.6</v>
@@ -2039,7 +2049,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>1747.1</v>
@@ -2098,7 +2108,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>2398.86386883434</v>
@@ -2157,7 +2167,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1679.23231807648</v>
@@ -2216,7 +2226,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1905.32218351584</v>
@@ -2275,7 +2285,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1968.88110515463</v>
@@ -2334,7 +2344,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>2708.71231090393</v>
@@ -2393,7 +2403,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>1903.58013454352</v>
@@ -2452,7 +2462,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>2209.94973449106</v>
@@ -2511,7 +2521,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>2161.65562016748</v>
@@ -2570,7 +2580,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>2845.82603759642</v>
@@ -2629,7 +2639,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>2074.47075910088</v>
@@ -2688,7 +2698,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>2220.49703180433</v>
@@ -2747,7 +2757,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>2157.68471807993</v>
@@ -2806,7 +2816,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2761.19404120798</v>
@@ -2865,7 +2875,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>1899.39115314154</v>
@@ -2924,7 +2934,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>2098.32520367766</v>
@@ -2983,7 +2993,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>2070.99836436598</v>
@@ -3042,7 +3052,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>2878.0472386878</v>
@@ -3101,7 +3111,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>2048.28319054732</v>
@@ -3160,7 +3170,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>2180.06020796427</v>
@@ -3219,7 +3229,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2112.86602822575</v>
@@ -3278,7 +3288,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>2935.63493973013</v>
@@ -3337,7 +3347,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>2085.81764439801</v>
@@ -3396,7 +3406,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>1894.04001281739</v>
@@ -3455,7 +3465,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1574.64834843281</v>
@@ -3514,7 +3524,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>1475.19763584073</v>
@@ -3573,7 +3583,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>1124.55064572027</v>
@@ -3632,7 +3642,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>1152.15904543455</v>
@@ -3691,7 +3701,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>1203.71436422561</v>
@@ -3750,7 +3760,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>1425.89524509937</v>
@@ -3809,7 +3819,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>1290.38528816145</v>
@@ -3868,7 +3878,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>1470.49652561565</v>
@@ -3927,7 +3937,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>1506.23806134637</v>
@@ -3986,7 +3996,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>1689.82206595359</v>
@@ -4045,7 +4055,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>1445.19764128156</v>
@@ -4104,7 +4114,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>1649.16622342598</v>
@@ -4163,7 +4173,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1834.94060897935</v>
@@ -4222,7 +4232,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>1933.00273454338</v>
@@ -4281,7 +4291,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>1888.09456688716</v>
@@ -4340,7 +4350,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>1827.0050126273</v>
@@ -4399,7 +4409,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>1977.85475412658</v>
@@ -4458,7 +4468,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>2160.36159801246</v>
@@ -4517,7 +4527,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>2033.21078101257</v>
@@ -4576,7 +4586,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>2167.47837936594</v>
@@ -4635,7 +4645,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>2312.92176137013</v>
@@ -4694,7 +4704,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>2696.86049566001</v>
@@ -4753,7 +4763,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>2516.13485121782</v>
@@ -4812,7 +4822,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>2803.88411969971</v>
@@ -4871,7 +4881,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>3010.33905330945</v>
@@ -4930,7 +4940,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>3500.76983696121</v>
@@ -4989,7 +4999,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>3286.26557559881</v>
@@ -5048,7 +5058,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>3537.71845126756</v>
@@ -5107,7 +5117,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>3321.73023465199</v>
@@ -5166,7 +5176,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>3386.00448971788</v>
@@ -5225,7 +5235,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>2696.05052423399</v>
@@ -5284,7 +5294,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>3036.48849479411</v>
@@ -5343,7 +5353,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>3418.10930449306</v>
@@ -5402,7 +5412,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>3735.59369195447</v>
@@ -5461,7 +5471,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>3551.93509050901</v>
@@ -5520,7 +5530,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>3501.98814428698</v>
@@ -5579,7 +5589,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>3831.21508377001</v>
@@ -5638,7 +5648,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>4375.22212253129</v>
@@ -5697,7 +5707,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>4129.41074094782</v>
@@ -5756,7 +5766,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>4333.19154339499</v>
@@ -5815,7 +5825,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>4811.64490558585</v>
@@ -5874,7 +5884,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>5066.12763917827</v>
@@ -5933,7 +5943,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>4383.03555041862</v>
@@ -5992,7 +6002,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>4429.87614408065</v>
@@ -6051,7 +6061,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>4465.28611985202</v>
@@ -6110,7 +6120,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>5131.88191643965</v>
@@ -6169,7 +6179,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>4499.44907972728</v>
@@ -6228,7 +6238,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>4539.76782551238</v>
@@ -6287,7 +6297,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>4837.70906203481</v>
@@ -6346,7 +6356,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>4964.35954377805</v>
@@ -6405,7 +6415,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>4294.14828388207</v>
@@ -6464,7 +6474,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>4320.30298531754</v>
@@ -6523,7 +6533,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>4458.85316814996</v>
@@ -6582,7 +6592,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>5009.75394783902</v>
@@ -6641,7 +6651,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>4294.11901736909</v>
@@ -6700,7 +6710,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>4771.89666477564</v>
@@ -6759,7 +6769,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>4952.78741323696</v>
@@ -6818,7 +6828,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>6108.57642446564</v>
@@ -6877,7 +6887,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>4881.31680020904</v>
@@ -6936,7 +6946,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>5446.86304040468</v>
@@ -6995,7 +7005,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>5439.60580468164</v>
@@ -7054,7 +7064,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>7098.31965039088</v>
@@ -7113,7 +7123,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>5694.02546550393</v>
@@ -7172,7 +7182,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>6209.22803193611</v>
@@ -7231,7 +7241,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>6200.06740637572</v>
@@ -7290,7 +7300,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>7870.36784763967</v>
@@ -7349,7 +7359,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>6054.57948367958</v>
@@ -7408,7 +7418,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>5310.71118746629</v>
@@ -7467,7 +7477,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>5041.77244509139</v>
@@ -7526,7 +7536,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>5651.60509658883</v>
@@ -7585,7 +7595,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>4665.68219017201</v>
@@ -7644,7 +7654,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>4755.00405694119</v>
@@ -7703,7 +7713,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>4573.30287832837</v>
@@ -7762,7 +7772,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>4670.88465711875</v>
@@ -7821,7 +7831,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>2175.26624692192</v>
@@ -7880,7 +7890,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>2405.16348217783</v>
@@ -7939,7 +7949,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>2776.70598703957</v>
@@ -7998,7 +8008,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>2640.35379506736</v>
@@ -8057,7 +8067,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>2885.42830497867</v>
@@ -8116,7 +8126,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>3444.49013745048</v>
@@ -8175,7 +8185,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>4318.55493831423</v>
@@ -8234,7 +8244,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>5038.84746379941</v>
@@ -8293,7 +8303,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>5155.69426033944</v>
@@ -8352,7 +8362,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>5721.03663102072</v>
@@ -8411,7 +8421,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>5275.14336147936</v>
@@ -8470,7 +8480,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>6464.88884607211</v>
@@ -8529,7 +8539,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>5373.68391411676</v>
@@ -8588,7 +8598,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>5519.15105764071</v>
@@ -8647,7 +8657,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>5214.52990895346</v>
@@ -8706,7 +8716,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>5530.3441739009</v>
@@ -8765,7 +8775,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>5009.70362811794</v>
@@ -8824,7 +8834,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>6033.85596798828</v>
@@ -8883,7 +8893,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>6342.86762614381</v>
@@ -8942,7 +8952,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>9133.82917570275</v>
@@ -9001,7 +9011,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>6663.08011470637</v>
@@ -9060,7 +9070,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>6896.80805983389</v>
@@ -9119,7 +9129,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>6578.69950141729</v>
@@ -9178,7 +9188,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2"/>
       <c r="C130" s="3" t="n">
@@ -9211,7 +9221,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2"/>
       <c r="C131" s="3" t="n">
@@ -9244,7 +9254,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2"/>
       <c r="C132" s="3" t="n">
@@ -9277,7 +9287,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2"/>
       <c r="C133" s="3" t="n">
@@ -9310,7 +9320,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2"/>
       <c r="C134" s="3"/>
@@ -9333,7 +9343,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2"/>
       <c r="C135" s="3"/>
@@ -9356,7 +9366,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2"/>
       <c r="C136" s="3"/>
@@ -9379,7 +9389,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2"/>
       <c r="C137" s="3"/>
@@ -9402,7 +9412,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2"/>
       <c r="C138" s="3"/>
@@ -9425,7 +9435,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2"/>
       <c r="C139" s="3"/>
@@ -9448,7 +9458,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2"/>
       <c r="C140" s="3"/>
@@ -9471,7 +9481,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2"/>
       <c r="C141" s="3"/>
@@ -9494,7 +9504,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2"/>
       <c r="C142" s="3"/>
@@ -9517,7 +9527,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2"/>
       <c r="C143" s="3"/>
@@ -9540,7 +9550,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2"/>
       <c r="C144" s="3"/>
@@ -9563,7 +9573,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2"/>
       <c r="C145" s="3"/>
@@ -9586,7 +9596,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2"/>
       <c r="C146" s="3"/>
@@ -9609,7 +9619,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2"/>
       <c r="C147" s="3"/>
@@ -9632,7 +9642,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2"/>
       <c r="C148" s="3"/>
@@ -9655,7 +9665,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2"/>
       <c r="C149" s="3"/>
@@ -9689,97 +9699,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -9803,7 +9813,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -9813,80 +9823,80 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0760360616958245</v>
+        <v>-0.0776990570851476</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0420889856838775</v>
+        <v>0.0439167477028377</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.226691643338528</v>
+        <v>0.22932987864076</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.437105690310537</v>
+        <v>0.436736073625052</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.579327025860819</v>
+        <v>0.577296261064304</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.561331652381918</v>
+        <v>0.560510095456793</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.404730761410807</v>
+        <v>0.406320642893262</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.215646368191768</v>
+        <v>0.218546449441727</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.0880231819730406</v>
+        <v>0.0893269871463753</v>
       </c>
     </row>
     <row r="14">

</xml_diff>